<commit_message>
New/Updated ontologies: aic and mns
</commit_message>
<xml_diff>
--- a/data/source/ontologies_source.xlsx
+++ b/data/source/ontologies_source.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fbosche\Documents\GitHub\BE-OLS\data\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D2634B8-686F-4910-8802-3E189E150250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1294C1-FAEB-4722-96F6-46089FB9F58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{C460B36E-D875-4E13-ACEB-9CF2004FB6B5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C460B36E-D875-4E13-ACEB-9CF2004FB6B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="14" r:id="rId1"/>
@@ -390,7 +390,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2743" uniqueCount="1085">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2757" uniqueCount="1092">
   <si>
     <t>BE Product (Building)</t>
   </si>
@@ -2655,9 +2655,6 @@
   </si>
   <si>
     <t>https://digiconstructlab-tu-delft.github.io/AiC-Ontology/</t>
-  </si>
-  <si>
-    <t>The Agents in Construction (AiC) ontology is a lightweight semantic model for coordinating on-site production in construction. It represents construction agents (human workers, robots, and other autonomous hardware) as they operate on a site: the processes they carry out, the elements they modify, the resources they handle, and the operational modes and metrics used to assess their performance and impact. To express how agent activities evolve over time, AiC introduces meta-properties that specify when a statement holds (at an instant or over an interval), what dimension of information it represents (planned, simulated, or performed), and who generated it. The ontology emphasizes generic, trade-agnostic concepts to ensure broad applicability across project types and delivery methods.</t>
   </si>
   <si>
     <t>dct</t>
@@ -3653,6 +3650,30 @@
   </si>
   <si>
     <t>This ontology provides a semantic framework for representing roof condition inspection information, including roofs and roof pitches, inspections, orthophotos, and image-derived defect observations. It is designed to support structured documentation, querying, and interoperability within digital twin–based workflows for roof condition monitoring and maintenance, particularly in the context of existing and heritage buildings.</t>
+  </si>
+  <si>
+    <t>The Agents in Construction (AiC) ontology is a lightweight semantic model for coordinating on-site production in construction. It represents construction agents (human workers, robots, and other autonomous hardware) and their state as they operate on a site: the processes they carry out, the elements they modify, the resources they handle, and the operational modes and metrics used to assess their performance and impact. To express how agents' operations evolve over time, AiC introduces meta-properties that specify when a statement holds (at an instant or over an interval), what dimension of information it represents (planned, simulated, or performed), and who generated it. The ontology emphasizes generic, trade-agnostic concepts to ensure broad applicability across project types and delivery methods.</t>
+  </si>
+  <si>
+    <t>Modelling and Standards Ontology</t>
+  </si>
+  <si>
+    <t>mns</t>
+  </si>
+  <si>
+    <t>https://w3id.org/mns#</t>
+  </si>
+  <si>
+    <t>https:\\doi.org\10.35490/EC3.2025.439</t>
+  </si>
+  <si>
+    <t>CC-BY-4.0</t>
+  </si>
+  <si>
+    <t>This ontology is developed to make the BIM Standards Landscape Explorer machine-readable on one hand, and also to create a connction between standards and other datasets and ontologies. This is a project from EC3 Modelling and Standards Committee. This is work-in-progress.</t>
+  </si>
+  <si>
+    <t>beo; bot; csite; cto; dica; dice; dicm; dicp; dtc; ioc; nen2660</t>
   </si>
 </sst>
 </file>
@@ -3944,8 +3965,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EFE1469B-541D-4DB3-969C-63DB4F642030}" name="Table2" displayName="Table2" ref="A1:V145" totalsRowShown="0" headerRowDxfId="14">
-  <autoFilter ref="A1:V145" xr:uid="{EFE1469B-541D-4DB3-969C-63DB4F642030}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EFE1469B-541D-4DB3-969C-63DB4F642030}" name="Table2" displayName="Table2" ref="A1:V146" totalsRowShown="0" headerRowDxfId="14">
+  <autoFilter ref="A1:V146" xr:uid="{EFE1469B-541D-4DB3-969C-63DB4F642030}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V145">
     <sortCondition ref="B1:B145"/>
   </sortState>
@@ -4362,7 +4383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6484B993-682B-477D-B31E-A58D58B7BF22}">
-  <dimension ref="A1:Z145"/>
+  <dimension ref="A1:Z146"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.5703125" customWidth="1"/>
@@ -4374,14 +4395,14 @@
     <col min="10" max="10" width="7" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="45.5703125" style="3" customWidth="1"/>
-    <col min="13" max="13" width="26.5703125" style="3" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="46" style="3" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="32.140625" style="32" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="26.5703125" style="3" customWidth="1"/>
+    <col min="14" max="14" width="46" style="3" customWidth="1"/>
+    <col min="15" max="15" width="32.140625" style="32" customWidth="1"/>
     <col min="16" max="16" width="26.140625" style="32" hidden="1" customWidth="1"/>
     <col min="17" max="17" width="21.42578125" style="32" hidden="1" customWidth="1"/>
     <col min="18" max="18" width="19.5703125" style="32" hidden="1" customWidth="1"/>
     <col min="19" max="19" width="19" style="32" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="0" style="30" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="8.85546875" style="30" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="36.42578125" style="30" customWidth="1"/>
     <col min="22" max="22" width="41.28515625" style="3" customWidth="1"/>
   </cols>
@@ -4403,7 +4424,7 @@
         <v>659</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="G1" s="22" t="s">
         <v>747</v>
@@ -4442,16 +4463,16 @@
         <v>743</v>
       </c>
       <c r="S1" s="26" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="T1" s="24" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="U1" s="22" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="V1" s="31" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="255" x14ac:dyDescent="0.25">
@@ -4510,13 +4531,13 @@
         <v>30</v>
       </c>
       <c r="U2" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>904</v>
-      </c>
-    </row>
-    <row r="3" spans="1:22" ht="105" x14ac:dyDescent="0.25">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" ht="270" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>751</v>
       </c>
@@ -4539,23 +4560,23 @@
         <v>14</v>
       </c>
       <c r="I3" s="28" t="s">
-        <v>241</v>
+        <v>393</v>
       </c>
       <c r="J3">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="K3" t="s">
         <v>133</v>
       </c>
       <c r="L3" s="3" t="s">
+        <v>1084</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>755</v>
       </c>
-      <c r="M3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>756</v>
-      </c>
       <c r="O3" s="32" t="s">
         <v>29</v>
       </c>
@@ -4572,10 +4593,10 @@
         <v>30</v>
       </c>
       <c r="U3" s="32" t="s">
+        <v>899</v>
+      </c>
+      <c r="V3" s="34" t="s">
         <v>900</v>
-      </c>
-      <c r="V3" s="34" t="s">
-        <v>901</v>
       </c>
     </row>
     <row r="4" spans="1:22" ht="165" x14ac:dyDescent="0.25">
@@ -4637,10 +4658,10 @@
         <v>15</v>
       </c>
       <c r="U4" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="195" x14ac:dyDescent="0.25">
@@ -4675,7 +4696,7 @@
         <v>35</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>36</v>
@@ -4699,10 +4720,10 @@
         <v>29</v>
       </c>
       <c r="U5" s="30" t="s">
+        <v>904</v>
+      </c>
+      <c r="V5" s="3" t="s">
         <v>905</v>
-      </c>
-      <c r="V5" s="3" t="s">
-        <v>906</v>
       </c>
     </row>
     <row r="6" spans="1:22" ht="150" x14ac:dyDescent="0.25">
@@ -4740,7 +4761,7 @@
         <v>23</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>38</v>
@@ -4767,10 +4788,10 @@
         <v>15</v>
       </c>
       <c r="U6" s="30" t="s">
+        <v>906</v>
+      </c>
+      <c r="V6" s="3" t="s">
         <v>907</v>
-      </c>
-      <c r="V6" s="3" t="s">
-        <v>908</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -4829,10 +4850,10 @@
         <v>30</v>
       </c>
       <c r="U7" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="210" x14ac:dyDescent="0.25">
@@ -4867,7 +4888,7 @@
         <v>38</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="M8" s="3" t="s">
         <v>38</v>
@@ -4891,10 +4912,10 @@
         <v>30</v>
       </c>
       <c r="U8" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V8" s="3" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="9" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -4929,7 +4950,7 @@
         <v>23</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>38</v>
@@ -4956,10 +4977,10 @@
         <v>22</v>
       </c>
       <c r="U9" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V9" s="3" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="60" x14ac:dyDescent="0.25">
@@ -4994,7 +5015,7 @@
         <v>57</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>38</v>
@@ -5021,10 +5042,10 @@
         <v>15</v>
       </c>
       <c r="U10" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V10" s="3" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -5083,10 +5104,10 @@
         <v>29</v>
       </c>
       <c r="U11" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V11" s="3" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -5142,10 +5163,10 @@
         <v>30</v>
       </c>
       <c r="U12" s="30" t="s">
+        <v>930</v>
+      </c>
+      <c r="V12" s="3" t="s">
         <v>931</v>
-      </c>
-      <c r="V12" s="3" t="s">
-        <v>932</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="255" x14ac:dyDescent="0.25">
@@ -5204,10 +5225,10 @@
         <v>15</v>
       </c>
       <c r="U13" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V13" s="3" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
     </row>
     <row r="14" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -5239,7 +5260,7 @@
         <v>38</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>72</v>
@@ -5266,10 +5287,10 @@
         <v>15</v>
       </c>
       <c r="U14" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V14" s="3" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
     </row>
     <row r="15" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -5304,7 +5325,7 @@
         <v>23</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>38</v>
@@ -5331,10 +5352,10 @@
         <v>15</v>
       </c>
       <c r="U15" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V15" s="3" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="16" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -5396,10 +5417,10 @@
         <v>30</v>
       </c>
       <c r="U16" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V16" s="3" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="17" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -5434,13 +5455,13 @@
         <v>85</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>38</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="O17" s="32" t="s">
         <v>29</v>
@@ -5458,10 +5479,10 @@
         <v>29</v>
       </c>
       <c r="U17" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V17" s="3" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="18" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -5472,7 +5493,7 @@
         <v>90</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="D18" t="s">
         <v>38</v>
@@ -5520,10 +5541,10 @@
         <v>29</v>
       </c>
       <c r="U18" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V18" s="3" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="19" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -5561,7 +5582,7 @@
         <v>98</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="M19" s="11" t="s">
         <v>100</v>
@@ -5588,10 +5609,10 @@
         <v>78</v>
       </c>
       <c r="U19" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V19" s="3" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="20" spans="1:22" ht="120" x14ac:dyDescent="0.25">
@@ -5650,10 +5671,10 @@
         <v>29</v>
       </c>
       <c r="U20" s="30" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="V20" s="3" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="21" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -5715,10 +5736,10 @@
         <v>15</v>
       </c>
       <c r="U21" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V21" s="3" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
     </row>
     <row r="22" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -5780,10 +5801,10 @@
         <v>30</v>
       </c>
       <c r="U22" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V22" s="3" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="23" spans="1:22" ht="270" x14ac:dyDescent="0.25">
@@ -5839,10 +5860,10 @@
         <v>29</v>
       </c>
       <c r="U23" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V23" s="3" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="24" spans="1:22" ht="225" x14ac:dyDescent="0.25">
@@ -5880,7 +5901,7 @@
         <v>38</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="M24" s="3" t="s">
         <v>122</v>
@@ -5904,10 +5925,10 @@
         <v>30</v>
       </c>
       <c r="U24" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V24" s="3" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="25" spans="1:22" ht="75" x14ac:dyDescent="0.25">
@@ -5945,7 +5966,7 @@
         <v>38</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>38</v>
@@ -5969,10 +5990,10 @@
         <v>30</v>
       </c>
       <c r="U25" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V25" s="3" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="75" x14ac:dyDescent="0.25">
@@ -6031,10 +6052,10 @@
         <v>29</v>
       </c>
       <c r="U26" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V26" s="3" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
     </row>
     <row r="27" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -6093,10 +6114,10 @@
         <v>29</v>
       </c>
       <c r="U27" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V27" s="3" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="28" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -6155,10 +6176,10 @@
         <v>29</v>
       </c>
       <c r="U28" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V28" s="3" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="29" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -6217,13 +6238,13 @@
         <v>29</v>
       </c>
       <c r="U29" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V29" s="3" t="s">
-        <v>949</v>
-      </c>
-    </row>
-    <row r="30" spans="1:22" ht="105" x14ac:dyDescent="0.25">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>584</v>
       </c>
@@ -6279,10 +6300,10 @@
         <v>30</v>
       </c>
       <c r="U30" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V30" s="3" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
     </row>
     <row r="31" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -6293,7 +6314,7 @@
         <v>132</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D31" t="s">
         <v>123</v>
@@ -6314,7 +6335,7 @@
         <v>133</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="M31" s="3" t="s">
         <v>135</v>
@@ -6338,10 +6359,10 @@
         <v>30</v>
       </c>
       <c r="U31" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V31" s="3" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
     </row>
     <row r="32" spans="1:22" ht="60" x14ac:dyDescent="0.25">
@@ -6352,7 +6373,7 @@
         <v>576</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="D32" t="s">
         <v>38</v>
@@ -6400,10 +6421,10 @@
         <v>30</v>
       </c>
       <c r="U32" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V32" s="3" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
     </row>
     <row r="33" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -6411,7 +6432,7 @@
         <v>137</v>
       </c>
       <c r="B33" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="C33" t="s">
         <v>38</v>
@@ -6441,7 +6462,7 @@
         <v>138</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="M33" s="3" t="s">
         <v>38</v>
@@ -6465,10 +6486,10 @@
         <v>29</v>
       </c>
       <c r="U33" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V33" s="3" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="34" spans="1:22" ht="75" x14ac:dyDescent="0.25">
@@ -6479,7 +6500,7 @@
         <v>143</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D34" t="s">
         <v>147</v>
@@ -6503,7 +6524,7 @@
         <v>23</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="M34" s="3" t="s">
         <v>145</v>
@@ -6527,10 +6548,10 @@
         <v>29</v>
       </c>
       <c r="U34" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V34" s="3" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="35" spans="1:22" ht="75" x14ac:dyDescent="0.25">
@@ -6541,7 +6562,7 @@
         <v>149</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="D35" t="s">
         <v>147</v>
@@ -6565,7 +6586,7 @@
         <v>133</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="N35" s="3" t="s">
         <v>151</v>
@@ -6586,10 +6607,10 @@
         <v>29</v>
       </c>
       <c r="U35" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V35" s="3" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="36" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -6600,7 +6621,7 @@
         <v>153</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="D36" t="s">
         <v>147</v>
@@ -6648,10 +6669,10 @@
         <v>29</v>
       </c>
       <c r="U36" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V36" s="3" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="37" spans="1:22" ht="75" x14ac:dyDescent="0.25">
@@ -6662,7 +6683,7 @@
         <v>159</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D37" t="s">
         <v>147</v>
@@ -6710,10 +6731,10 @@
         <v>30</v>
       </c>
       <c r="U37" s="30" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="V37" s="3" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="38" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -6724,7 +6745,7 @@
         <v>164</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="D38" t="s">
         <v>147</v>
@@ -6772,10 +6793,10 @@
         <v>29</v>
       </c>
       <c r="U38" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V38" s="3" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
     </row>
     <row r="39" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -6786,7 +6807,7 @@
         <v>169</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="D39" t="s">
         <v>147</v>
@@ -6810,7 +6831,7 @@
         <v>133</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>167</v>
@@ -6834,10 +6855,10 @@
         <v>30</v>
       </c>
       <c r="U39" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V39" s="3" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
     </row>
     <row r="40" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -6867,7 +6888,7 @@
         <v>38</v>
       </c>
       <c r="L40" s="3" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="M40" s="3" t="s">
         <v>38</v>
@@ -6891,13 +6912,13 @@
         <v>30</v>
       </c>
       <c r="U40" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V40" s="3" t="s">
-        <v>966</v>
-      </c>
-    </row>
-    <row r="41" spans="1:22" ht="90" x14ac:dyDescent="0.25">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" ht="105" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>172</v>
       </c>
@@ -6905,7 +6926,7 @@
         <v>173</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="D41" t="s">
         <v>147</v>
@@ -6953,13 +6974,13 @@
         <v>29</v>
       </c>
       <c r="U41" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V41" s="3" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="42" spans="1:22" ht="105" x14ac:dyDescent="0.25">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" ht="180" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>177</v>
       </c>
@@ -6967,7 +6988,7 @@
         <v>178</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="D42" t="s">
         <v>147</v>
@@ -7018,10 +7039,10 @@
         <v>30</v>
       </c>
       <c r="U42" s="30" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="V42" s="3" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
     </row>
     <row r="43" spans="1:22" ht="300" x14ac:dyDescent="0.25">
@@ -7032,7 +7053,7 @@
         <v>183</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="D43" t="s">
         <v>147</v>
@@ -7080,10 +7101,10 @@
         <v>29</v>
       </c>
       <c r="U43" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V43" s="3" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="44" spans="1:22" ht="255" x14ac:dyDescent="0.25">
@@ -7094,7 +7115,7 @@
         <v>188</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D44" t="s">
         <v>147</v>
@@ -7107,7 +7128,7 @@
         <v>14</v>
       </c>
       <c r="L44" s="3" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="M44" s="3" t="s">
         <v>38</v>
@@ -7131,10 +7152,10 @@
         <v>30</v>
       </c>
       <c r="U44" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V44" s="3" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="45" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -7145,7 +7166,7 @@
         <v>190</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="D45" t="s">
         <v>147</v>
@@ -7167,7 +7188,7 @@
         <v>133</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>38</v>
@@ -7191,10 +7212,10 @@
         <v>29</v>
       </c>
       <c r="U45" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V45" s="3" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="46" spans="1:22" ht="165" x14ac:dyDescent="0.25">
@@ -7205,7 +7226,7 @@
         <v>192</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="D46" t="s">
         <v>147</v>
@@ -7253,10 +7274,10 @@
         <v>29</v>
       </c>
       <c r="U46" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V46" s="3" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="47" spans="1:22" ht="285" x14ac:dyDescent="0.25">
@@ -7294,7 +7315,7 @@
         <v>38</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>38</v>
@@ -7318,10 +7339,10 @@
         <v>30</v>
       </c>
       <c r="U47" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V47" s="3" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="48" spans="1:22" ht="120" x14ac:dyDescent="0.25">
@@ -7359,7 +7380,7 @@
         <v>38</v>
       </c>
       <c r="L48" s="3" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="M48" s="3" t="s">
         <v>38</v>
@@ -7383,13 +7404,13 @@
         <v>30</v>
       </c>
       <c r="U48" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V48" s="3" t="s">
-        <v>959</v>
-      </c>
-    </row>
-    <row r="49" spans="1:22" ht="180" x14ac:dyDescent="0.25">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" ht="105" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>198</v>
       </c>
@@ -7397,7 +7418,7 @@
         <v>199</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="D49" t="s">
         <v>38</v>
@@ -7442,10 +7463,10 @@
         <v>30</v>
       </c>
       <c r="U49" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V49" s="3" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="50" spans="1:22" ht="60" x14ac:dyDescent="0.25">
@@ -7483,7 +7504,7 @@
         <v>23</v>
       </c>
       <c r="L50" s="3" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="M50" s="3" t="s">
         <v>208</v>
@@ -7507,10 +7528,10 @@
         <v>30</v>
       </c>
       <c r="U50" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V50" s="3" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="51" spans="1:22" ht="75" x14ac:dyDescent="0.25">
@@ -7572,13 +7593,13 @@
         <v>30</v>
       </c>
       <c r="U51" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V51" s="3" t="s">
-        <v>956</v>
-      </c>
-    </row>
-    <row r="52" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="52" spans="1:22" ht="105" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>214</v>
       </c>
@@ -7613,7 +7634,7 @@
         <v>38</v>
       </c>
       <c r="L52" s="3" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="M52" s="3" t="s">
         <v>218</v>
@@ -7637,10 +7658,10 @@
         <v>30</v>
       </c>
       <c r="U52" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V52" s="3" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="53" spans="1:22" ht="360" x14ac:dyDescent="0.25">
@@ -7699,27 +7720,27 @@
         <v>30</v>
       </c>
       <c r="U53" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V53" s="3" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="54" spans="1:22" ht="90" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>757</v>
+      </c>
+      <c r="B54" t="s">
         <v>758</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" s="1" t="s">
         <v>759</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="D54" t="s">
+        <v>38</v>
+      </c>
+      <c r="E54" t="s">
         <v>760</v>
-      </c>
-      <c r="D54" t="s">
-        <v>38</v>
-      </c>
-      <c r="E54" t="s">
-        <v>761</v>
       </c>
       <c r="G54" t="s">
         <v>609</v>
@@ -7734,14 +7755,14 @@
         <v>248</v>
       </c>
       <c r="L54" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="M54" s="3" t="s">
         <v>762</v>
       </c>
-      <c r="M54" s="3" t="s">
+      <c r="N54" s="3" t="s">
         <v>763</v>
       </c>
-      <c r="N54" s="3" t="s">
-        <v>764</v>
-      </c>
       <c r="O54" s="32" t="s">
         <v>29</v>
       </c>
@@ -7758,10 +7779,10 @@
         <v>30</v>
       </c>
       <c r="U54" s="32" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V54" s="34" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="55" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -7796,7 +7817,7 @@
         <v>231</v>
       </c>
       <c r="L55" s="3" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="M55" s="3" t="s">
         <v>38</v>
@@ -7820,10 +7841,10 @@
         <v>30</v>
       </c>
       <c r="U55" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V55" s="3" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
     </row>
     <row r="56" spans="1:22" ht="135" x14ac:dyDescent="0.25">
@@ -7834,7 +7855,7 @@
         <v>235</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D56" t="s">
         <v>38</v>
@@ -7858,7 +7879,7 @@
         <v>237</v>
       </c>
       <c r="L56" s="3" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="M56" s="3" t="s">
         <v>38</v>
@@ -7882,10 +7903,10 @@
         <v>30</v>
       </c>
       <c r="U56" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V56" s="3" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="57" spans="1:22" ht="180" x14ac:dyDescent="0.25">
@@ -7947,10 +7968,10 @@
         <v>30</v>
       </c>
       <c r="U57" s="30" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="V57" s="3" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="58" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -7985,7 +8006,7 @@
         <v>248</v>
       </c>
       <c r="L58" s="3" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="M58" s="3" t="s">
         <v>38</v>
@@ -8009,13 +8030,13 @@
         <v>30</v>
       </c>
       <c r="U58" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V58" s="3" t="s">
-        <v>982</v>
-      </c>
-    </row>
-    <row r="59" spans="1:22" ht="135" x14ac:dyDescent="0.25">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="59" spans="1:22" ht="105" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>251</v>
       </c>
@@ -8047,7 +8068,7 @@
         <v>23</v>
       </c>
       <c r="L59" s="3" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="M59" s="3" t="s">
         <v>256</v>
@@ -8071,10 +8092,10 @@
         <v>29</v>
       </c>
       <c r="U59" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V59" s="3" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="60" spans="1:22" ht="180" x14ac:dyDescent="0.25">
@@ -8085,7 +8106,7 @@
         <v>258</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="D60" t="s">
         <v>38</v>
@@ -8109,7 +8130,7 @@
         <v>260</v>
       </c>
       <c r="L60" s="3" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="M60" s="3" t="s">
         <v>38</v>
@@ -8133,10 +8154,10 @@
         <v>30</v>
       </c>
       <c r="U60" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V60" s="3" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
     </row>
     <row r="61" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -8144,7 +8165,7 @@
         <v>652</v>
       </c>
       <c r="B61" s="17" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C61" s="17" t="s">
         <v>38</v>
@@ -8172,7 +8193,7 @@
         <v>653</v>
       </c>
       <c r="L61" s="3" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="M61" s="15" t="s">
         <v>38</v>
@@ -8196,10 +8217,10 @@
         <v>30</v>
       </c>
       <c r="U61" s="30" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="V61" s="3" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
     </row>
     <row r="62" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -8258,10 +8279,10 @@
         <v>30</v>
       </c>
       <c r="U62" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V62" s="3" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
     </row>
     <row r="63" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -8323,27 +8344,27 @@
         <v>30</v>
       </c>
       <c r="U63" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V63" s="3" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
     </row>
     <row r="64" spans="1:22" ht="180" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>764</v>
+      </c>
+      <c r="B64" t="s">
         <v>765</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" s="1" t="s">
         <v>766</v>
       </c>
-      <c r="C64" s="1" t="s">
+      <c r="D64" t="s">
+        <v>38</v>
+      </c>
+      <c r="E64" s="1" t="s">
         <v>767</v>
-      </c>
-      <c r="D64" t="s">
-        <v>38</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>768</v>
       </c>
       <c r="G64" t="s">
         <v>15</v>
@@ -8361,13 +8382,13 @@
         <v>35</v>
       </c>
       <c r="L64" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="M64" s="3" t="s">
         <v>769</v>
       </c>
-      <c r="M64" s="3" t="s">
-        <v>770</v>
-      </c>
       <c r="N64" s="3" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="O64" s="32" t="s">
         <v>29</v>
@@ -8385,10 +8406,10 @@
         <v>30</v>
       </c>
       <c r="U64" s="32" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V64" s="34" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="65" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -8447,10 +8468,10 @@
         <v>29</v>
       </c>
       <c r="U65" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V65" s="3" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
     </row>
     <row r="66" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -8488,7 +8509,7 @@
         <v>23</v>
       </c>
       <c r="L66" s="3" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="M66" s="3" t="s">
         <v>83</v>
@@ -8512,10 +8533,10 @@
         <v>29</v>
       </c>
       <c r="U66" s="30" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="V66" s="3" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
     </row>
     <row r="67" spans="1:22" ht="210" x14ac:dyDescent="0.25">
@@ -8553,7 +8574,7 @@
         <v>38</v>
       </c>
       <c r="L67" s="3" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="M67" s="3" t="s">
         <v>38</v>
@@ -8577,10 +8598,10 @@
         <v>30</v>
       </c>
       <c r="U67" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V67" s="3" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
     </row>
     <row r="68" spans="1:22" ht="180" x14ac:dyDescent="0.25">
@@ -8618,7 +8639,7 @@
         <v>38</v>
       </c>
       <c r="L68" s="3" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="M68" s="3" t="s">
         <v>38</v>
@@ -8642,10 +8663,10 @@
         <v>30</v>
       </c>
       <c r="U68" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V68" s="3" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
     </row>
     <row r="69" spans="1:22" ht="409.5" x14ac:dyDescent="0.25">
@@ -8656,7 +8677,7 @@
         <v>665</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="D69" t="s">
         <v>38</v>
@@ -8680,7 +8701,7 @@
         <v>582</v>
       </c>
       <c r="L69" s="3" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="N69" s="11"/>
       <c r="O69" s="32" t="s">
@@ -8699,10 +8720,10 @@
         <v>29</v>
       </c>
       <c r="U69" s="30" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="V69" s="3" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
     </row>
     <row r="70" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -8710,7 +8731,7 @@
         <v>502</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="C70" s="17" t="s">
         <v>38</v>
@@ -8762,10 +8783,10 @@
       </c>
       <c r="T70" s="32"/>
       <c r="U70" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V70" s="3" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
     </row>
     <row r="71" spans="1:22" ht="120" x14ac:dyDescent="0.25">
@@ -8773,7 +8794,7 @@
         <v>539</v>
       </c>
       <c r="B71" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C71" s="9" t="s">
         <v>38</v>
@@ -8824,27 +8845,27 @@
         <v>30</v>
       </c>
       <c r="U71" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V71" s="3" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
     </row>
     <row r="72" spans="1:22" ht="105" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>771</v>
+      </c>
+      <c r="B72" t="s">
         <v>772</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" s="1" t="s">
         <v>773</v>
       </c>
-      <c r="C72" s="1" t="s">
+      <c r="D72" t="s">
+        <v>38</v>
+      </c>
+      <c r="E72" s="1" t="s">
         <v>774</v>
-      </c>
-      <c r="D72" t="s">
-        <v>38</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>775</v>
       </c>
       <c r="G72" t="s">
         <v>0</v>
@@ -8862,14 +8883,14 @@
         <v>35</v>
       </c>
       <c r="L72" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="M72" s="3" t="s">
         <v>776</v>
       </c>
-      <c r="M72" s="3" t="s">
+      <c r="N72" s="3" t="s">
         <v>777</v>
       </c>
-      <c r="N72" s="3" t="s">
-        <v>778</v>
-      </c>
       <c r="O72" s="32" t="s">
         <v>29</v>
       </c>
@@ -8886,10 +8907,10 @@
         <v>29</v>
       </c>
       <c r="U72" s="32" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V72" s="34" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="73" spans="1:22" ht="165" x14ac:dyDescent="0.25">
@@ -8927,7 +8948,7 @@
         <v>23</v>
       </c>
       <c r="L73" s="3" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="M73" s="3" t="s">
         <v>278</v>
@@ -8954,10 +8975,10 @@
         <v>0</v>
       </c>
       <c r="U73" s="30" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="V73" s="3" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
     </row>
     <row r="74" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -8992,7 +9013,7 @@
         <v>23</v>
       </c>
       <c r="L74" s="3" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M74" s="3" t="s">
         <v>509</v>
@@ -9016,10 +9037,10 @@
         <v>30</v>
       </c>
       <c r="U74" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V74" s="3" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
     </row>
     <row r="75" spans="1:22" ht="75" x14ac:dyDescent="0.25">
@@ -9030,7 +9051,7 @@
         <v>507</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="D75" t="s">
         <v>38</v>
@@ -9057,7 +9078,7 @@
         <v>248</v>
       </c>
       <c r="L75" s="3" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="M75" s="3" t="s">
         <v>38</v>
@@ -9082,10 +9103,10 @@
       </c>
       <c r="T75" s="39"/>
       <c r="U75" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V75" s="3" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
     </row>
     <row r="76" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -9096,7 +9117,7 @@
         <v>288</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="D76" t="s">
         <v>38</v>
@@ -9120,7 +9141,7 @@
         <v>35</v>
       </c>
       <c r="L76" s="3" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="M76" s="3" t="s">
         <v>38</v>
@@ -9144,10 +9165,10 @@
         <v>30</v>
       </c>
       <c r="U76" s="30" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="V76" s="3" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
     </row>
     <row r="77" spans="1:22" ht="120" x14ac:dyDescent="0.25">
@@ -9182,7 +9203,7 @@
         <v>23</v>
       </c>
       <c r="L77" s="3" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="M77" s="3" t="s">
         <v>38</v>
@@ -9209,10 +9230,10 @@
         <v>15</v>
       </c>
       <c r="U77" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V77" s="3" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="78" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -9223,7 +9244,7 @@
         <v>218</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="D78" t="s">
         <v>38</v>
@@ -9247,7 +9268,7 @@
         <v>231</v>
       </c>
       <c r="L78" s="3" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="M78" s="3" t="s">
         <v>296</v>
@@ -9271,10 +9292,10 @@
         <v>30</v>
       </c>
       <c r="U78" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V78" s="3" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
     </row>
     <row r="79" spans="1:22" ht="255" x14ac:dyDescent="0.25">
@@ -9333,10 +9354,10 @@
         <v>29</v>
       </c>
       <c r="U79" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V79" s="3" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="80" spans="1:22" ht="255" x14ac:dyDescent="0.25">
@@ -9362,7 +9383,7 @@
         <v>38</v>
       </c>
       <c r="L80" s="3" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="M80" s="3" t="s">
         <v>306</v>
@@ -9386,13 +9407,13 @@
         <v>29</v>
       </c>
       <c r="U80" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V80" s="3" t="s">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="81" spans="1:22" ht="409.5" x14ac:dyDescent="0.25">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="81" spans="1:22" ht="165" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>510</v>
       </c>
@@ -9429,10 +9450,10 @@
       <c r="N81" s="11"/>
       <c r="S81" s="33"/>
       <c r="U81" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V81" s="3" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="82" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -9491,10 +9512,10 @@
         <v>29</v>
       </c>
       <c r="U82" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V82" s="3" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="83" spans="1:22" ht="135" x14ac:dyDescent="0.25">
@@ -9532,7 +9553,7 @@
         <v>57</v>
       </c>
       <c r="L83" s="3" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="M83" s="3" t="s">
         <v>38</v>
@@ -9556,10 +9577,10 @@
         <v>30</v>
       </c>
       <c r="U83" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V83" s="3" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="84" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -9594,7 +9615,7 @@
         <v>23</v>
       </c>
       <c r="L84" s="3" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="M84" s="3" t="s">
         <v>38</v>
@@ -9618,10 +9639,10 @@
         <v>29</v>
       </c>
       <c r="U84" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V84" s="3" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="85" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -9680,10 +9701,10 @@
         <v>30</v>
       </c>
       <c r="U85" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V85" s="3" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
     </row>
     <row r="86" spans="1:22" s="17" customFormat="1" ht="165" x14ac:dyDescent="0.25">
@@ -9744,10 +9765,10 @@
       </c>
       <c r="T86" s="30"/>
       <c r="U86" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V86" s="3" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="87" spans="1:22" ht="225" x14ac:dyDescent="0.25">
@@ -9806,10 +9827,10 @@
         <v>30</v>
       </c>
       <c r="U87" s="30" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="V87" s="3" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="88" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -9868,10 +9889,10 @@
         <v>30</v>
       </c>
       <c r="U88" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V88" s="3" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="89" spans="1:22" ht="75" x14ac:dyDescent="0.25">
@@ -9933,10 +9954,10 @@
         <v>29</v>
       </c>
       <c r="U89" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V89" s="3" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="90" spans="1:22" ht="255" x14ac:dyDescent="0.25">
@@ -9971,7 +9992,7 @@
         <v>38</v>
       </c>
       <c r="L90" s="3" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="M90" s="3" t="s">
         <v>83</v>
@@ -9995,10 +10016,10 @@
         <v>30</v>
       </c>
       <c r="U90" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V90" s="3" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="91" spans="1:22" ht="165" x14ac:dyDescent="0.25">
@@ -10057,10 +10078,10 @@
         <v>29</v>
       </c>
       <c r="U91" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V91" s="3" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="92" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -10095,7 +10116,7 @@
         <v>23</v>
       </c>
       <c r="L92" s="3" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="M92" s="3" t="s">
         <v>38</v>
@@ -10119,10 +10140,10 @@
         <v>29</v>
       </c>
       <c r="U92" s="30" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="V92" s="3" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="93" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -10133,7 +10154,7 @@
         <v>272</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="D93" t="s">
         <v>38</v>
@@ -10181,10 +10202,10 @@
         <v>29</v>
       </c>
       <c r="U93" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V93" s="3" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="94" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -10219,7 +10240,7 @@
         <v>38</v>
       </c>
       <c r="L94" s="3" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="M94" s="3" t="s">
         <v>38</v>
@@ -10243,10 +10264,10 @@
         <v>30</v>
       </c>
       <c r="U94" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V94" s="3" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="95" spans="1:22" ht="105" x14ac:dyDescent="0.25">
@@ -10281,7 +10302,7 @@
         <v>38</v>
       </c>
       <c r="L95" s="3" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="M95" s="3" t="s">
         <v>38</v>
@@ -10305,10 +10326,10 @@
         <v>29</v>
       </c>
       <c r="U95" s="30" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="V95" s="3" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="96" spans="1:22" ht="150" x14ac:dyDescent="0.25">
@@ -10343,7 +10364,7 @@
         <v>38</v>
       </c>
       <c r="L96" s="3" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="M96" s="3" t="s">
         <v>38</v>
@@ -10367,10 +10388,10 @@
         <v>30</v>
       </c>
       <c r="U96" s="30" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="V96" s="3" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
     </row>
     <row r="97" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -10429,10 +10450,10 @@
         <v>30</v>
       </c>
       <c r="U97" s="30" t="s">
+        <v>919</v>
+      </c>
+      <c r="V97" s="3" t="s">
         <v>920</v>
-      </c>
-      <c r="V97" s="3" t="s">
-        <v>921</v>
       </c>
     </row>
     <row r="98" spans="1:26" ht="75" x14ac:dyDescent="0.25">
@@ -10491,27 +10512,27 @@
         <v>29</v>
       </c>
       <c r="U98" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V98" s="3" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="99" spans="1:26" ht="135" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>832</v>
+      </c>
+      <c r="B99" t="s">
         <v>833</v>
       </c>
-      <c r="B99" t="s">
+      <c r="C99" s="27" t="s">
         <v>834</v>
       </c>
-      <c r="C99" s="27" t="s">
+      <c r="D99" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E99" s="1" t="s">
         <v>835</v>
-      </c>
-      <c r="D99" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E99" s="1" t="s">
-        <v>836</v>
       </c>
       <c r="F99" t="s">
         <v>38</v>
@@ -10521,16 +10542,16 @@
       </c>
       <c r="H99" s="1"/>
       <c r="I99" s="10" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="J99">
         <v>2025</v>
       </c>
       <c r="K99" t="s">
+        <v>837</v>
+      </c>
+      <c r="L99" s="3" t="s">
         <v>838</v>
-      </c>
-      <c r="L99" s="3" t="s">
-        <v>839</v>
       </c>
       <c r="M99" s="3" t="s">
         <v>38</v>
@@ -10555,10 +10576,10 @@
       </c>
       <c r="T99" s="32"/>
       <c r="U99" s="32" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="V99" s="34" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="100" spans="1:26" ht="105" x14ac:dyDescent="0.25">
@@ -10593,7 +10614,7 @@
         <v>23</v>
       </c>
       <c r="L100" s="3" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="M100" s="3" t="s">
         <v>377</v>
@@ -10617,10 +10638,10 @@
         <v>29</v>
       </c>
       <c r="U100" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V100" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="101" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -10655,7 +10676,7 @@
         <v>23</v>
       </c>
       <c r="L101" s="3" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="M101" s="3" t="s">
         <v>382</v>
@@ -10679,27 +10700,27 @@
         <v>30</v>
       </c>
       <c r="U101" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V101" s="3" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="102" spans="1:26" ht="150" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
+        <v>1080</v>
+      </c>
+      <c r="B102" t="s">
         <v>1081</v>
       </c>
-      <c r="B102" t="s">
+      <c r="C102" s="41" t="s">
         <v>1082</v>
       </c>
-      <c r="C102" s="41" t="s">
-        <v>1083</v>
-      </c>
       <c r="D102" s="7" t="s">
         <v>38</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="F102" s="29" t="s">
         <v>38</v>
@@ -10720,7 +10741,7 @@
         <v>133</v>
       </c>
       <c r="L102" s="3" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="N102" s="11"/>
       <c r="S102" s="33"/>
@@ -10760,7 +10781,7 @@
         <v>385</v>
       </c>
       <c r="L103" s="3" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M103" s="3" t="s">
         <v>387</v>
@@ -10784,13 +10805,13 @@
         <v>29</v>
       </c>
       <c r="U103" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V103" s="3" t="s">
-        <v>1014</v>
-      </c>
-    </row>
-    <row r="104" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="104" spans="1:26" ht="285" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>600</v>
       </c>
@@ -10843,13 +10864,13 @@
         <v>30</v>
       </c>
       <c r="U104" s="30" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="V104" s="3" t="s">
-        <v>1015</v>
-      </c>
-    </row>
-    <row r="105" spans="1:26" ht="165" x14ac:dyDescent="0.25">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="105" spans="1:26" ht="195" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>389</v>
       </c>
@@ -10881,7 +10902,7 @@
         <v>57</v>
       </c>
       <c r="L105" s="3" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="M105" s="3" t="s">
         <v>38</v>
@@ -10905,10 +10926,10 @@
         <v>30</v>
       </c>
       <c r="U105" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V105" s="3" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="106" spans="1:26" ht="105" x14ac:dyDescent="0.25">
@@ -10943,7 +10964,7 @@
         <v>23</v>
       </c>
       <c r="L106" s="3" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="M106" s="3" t="s">
         <v>395</v>
@@ -10967,10 +10988,10 @@
         <v>30</v>
       </c>
       <c r="U106" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V106" s="3" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
     </row>
     <row r="107" spans="1:26" ht="90" x14ac:dyDescent="0.25">
@@ -11005,7 +11026,7 @@
         <v>23</v>
       </c>
       <c r="L107" s="3" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="M107" s="3" t="s">
         <v>401</v>
@@ -11029,13 +11050,13 @@
         <v>29</v>
       </c>
       <c r="U107" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V107" s="3" t="s">
-        <v>945</v>
-      </c>
-    </row>
-    <row r="108" spans="1:26" ht="120" x14ac:dyDescent="0.25">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="108" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>419</v>
       </c>
@@ -11067,7 +11088,7 @@
         <v>23</v>
       </c>
       <c r="L108" s="3" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="M108" s="3" t="s">
         <v>423</v>
@@ -11091,13 +11112,13 @@
         <v>30</v>
       </c>
       <c r="U108" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V108" s="3" t="s">
-        <v>946</v>
-      </c>
-    </row>
-    <row r="109" spans="1:26" ht="60" x14ac:dyDescent="0.25">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="109" spans="1:26" ht="165" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>424</v>
       </c>
@@ -11105,7 +11126,7 @@
         <v>425</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D109" t="s">
         <v>38</v>
@@ -11153,13 +11174,13 @@
         <v>30</v>
       </c>
       <c r="U109" s="30" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="V109" s="3" t="s">
-        <v>1037</v>
-      </c>
-    </row>
-    <row r="110" spans="1:26" ht="105" x14ac:dyDescent="0.25">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="110" spans="1:26" ht="75" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>430</v>
       </c>
@@ -11215,18 +11236,18 @@
         <v>29</v>
       </c>
       <c r="U110" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V110" s="3" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="111" spans="1:26" ht="165" x14ac:dyDescent="0.25">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="111" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A111" s="17" t="s">
         <v>633</v>
       </c>
       <c r="B111" s="17" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="C111" s="19" t="s">
         <v>634</v>
@@ -11254,7 +11275,7 @@
         <v>98</v>
       </c>
       <c r="L111" s="3" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="M111" s="15" t="s">
         <v>635</v>
@@ -11278,22 +11299,22 @@
         <v>30</v>
       </c>
       <c r="U111" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V111" s="3" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="Z111" s="3"/>
     </row>
-    <row r="112" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:26" ht="150" x14ac:dyDescent="0.25">
       <c r="A112" s="17" t="s">
         <v>637</v>
       </c>
       <c r="B112" s="17" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C112" s="19" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="D112" s="20" t="s">
         <v>405</v>
@@ -11320,7 +11341,7 @@
         <v>98</v>
       </c>
       <c r="L112" s="3" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="M112" s="15" t="s">
         <v>639</v>
@@ -11344,18 +11365,18 @@
         <v>30</v>
       </c>
       <c r="U112" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V112" s="3" t="s">
-        <v>1020</v>
-      </c>
-    </row>
-    <row r="113" spans="1:22" ht="135" x14ac:dyDescent="0.25">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="113" spans="1:22" ht="285" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>623</v>
       </c>
       <c r="B113" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="C113" s="2" t="s">
         <v>403</v>
@@ -11385,7 +11406,7 @@
         <v>98</v>
       </c>
       <c r="L113" s="3" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="M113" s="3" t="s">
         <v>404</v>
@@ -11409,21 +11430,21 @@
         <v>29</v>
       </c>
       <c r="U113" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V113" s="3" t="s">
-        <v>1021</v>
-      </c>
-    </row>
-    <row r="114" spans="1:22" ht="105" x14ac:dyDescent="0.25">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="114" spans="1:22" ht="90" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>625</v>
       </c>
       <c r="B114" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="D114" t="s">
         <v>405</v>
@@ -11450,7 +11471,7 @@
         <v>98</v>
       </c>
       <c r="L114" s="3" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="M114" s="3" t="s">
         <v>404</v>
@@ -11474,21 +11495,21 @@
         <v>29</v>
       </c>
       <c r="U114" s="30" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="V114" s="3" t="s">
-        <v>1028</v>
-      </c>
-    </row>
-    <row r="115" spans="1:22" ht="285" x14ac:dyDescent="0.25">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="115" spans="1:22" ht="255" x14ac:dyDescent="0.25">
       <c r="A115" s="17" t="s">
         <v>641</v>
       </c>
       <c r="B115" s="17" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="C115" s="19" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="D115" s="20" t="s">
         <v>405</v>
@@ -11513,7 +11534,7 @@
         <v>98</v>
       </c>
       <c r="L115" s="3" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="M115" s="15" t="s">
         <v>643</v>
@@ -11537,21 +11558,21 @@
         <v>30</v>
       </c>
       <c r="U115" s="30" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="V115" s="3" t="s">
-        <v>1023</v>
-      </c>
-    </row>
-    <row r="116" spans="1:22" ht="195" x14ac:dyDescent="0.25">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="116" spans="1:22" ht="135" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>624</v>
       </c>
       <c r="B116" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D116" t="s">
         <v>405</v>
@@ -11578,7 +11599,7 @@
         <v>98</v>
       </c>
       <c r="L116" s="3" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="M116" s="3" t="s">
         <v>404</v>
@@ -11602,10 +11623,10 @@
         <v>30</v>
       </c>
       <c r="U116" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V116" s="3" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="117" spans="1:22" ht="120" x14ac:dyDescent="0.25">
@@ -11613,10 +11634,10 @@
         <v>629</v>
       </c>
       <c r="B117" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="D117" t="s">
         <v>405</v>
@@ -11643,7 +11664,7 @@
         <v>98</v>
       </c>
       <c r="L117" s="3" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="M117" s="3" t="s">
         <v>404</v>
@@ -11667,21 +11688,21 @@
         <v>30</v>
       </c>
       <c r="U117" s="30" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="V117" s="3" t="s">
-        <v>1025</v>
-      </c>
-    </row>
-    <row r="118" spans="1:22" ht="300" x14ac:dyDescent="0.25">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="118" spans="1:22" ht="105" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>628</v>
       </c>
       <c r="B118" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="D118" t="s">
         <v>405</v>
@@ -11708,7 +11729,7 @@
         <v>98</v>
       </c>
       <c r="L118" s="3" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="M118" s="3" t="s">
         <v>404</v>
@@ -11732,21 +11753,21 @@
         <v>30</v>
       </c>
       <c r="U118" s="30" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="V118" s="3" t="s">
-        <v>1029</v>
-      </c>
-    </row>
-    <row r="119" spans="1:22" ht="270" x14ac:dyDescent="0.25">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="119" spans="1:22" ht="120" x14ac:dyDescent="0.25">
       <c r="A119" s="17" t="s">
         <v>645</v>
       </c>
       <c r="B119" s="17" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="C119" s="19" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D119" s="20" t="s">
         <v>405</v>
@@ -11773,7 +11794,7 @@
         <v>98</v>
       </c>
       <c r="L119" s="3" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="M119" s="15" t="s">
         <v>404</v>
@@ -11797,21 +11818,21 @@
         <v>30</v>
       </c>
       <c r="U119" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V119" s="3" t="s">
-        <v>1026</v>
-      </c>
-    </row>
-    <row r="120" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="120" spans="1:22" ht="90" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>627</v>
       </c>
       <c r="B120" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="D120" t="s">
         <v>405</v>
@@ -11838,7 +11859,7 @@
         <v>98</v>
       </c>
       <c r="L120" s="3" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="M120" s="3" t="s">
         <v>413</v>
@@ -11862,21 +11883,21 @@
         <v>30</v>
       </c>
       <c r="U120" s="30" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="V120" s="3" t="s">
-        <v>1030</v>
-      </c>
-    </row>
-    <row r="121" spans="1:22" ht="150" x14ac:dyDescent="0.25">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="121" spans="1:22" ht="60" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>631</v>
       </c>
       <c r="B121" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D121" t="s">
         <v>405</v>
@@ -11924,18 +11945,18 @@
         <v>29</v>
       </c>
       <c r="U121" s="30" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="V121" s="3" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="122" spans="1:22" s="17" customFormat="1" ht="285" x14ac:dyDescent="0.25">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="122" spans="1:22" s="17" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>626</v>
       </c>
       <c r="B122" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="C122" s="2" t="s">
         <v>418</v>
@@ -11965,7 +11986,7 @@
         <v>98</v>
       </c>
       <c r="L122" s="3" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="M122" s="3" t="s">
         <v>632</v>
@@ -11990,21 +12011,21 @@
       </c>
       <c r="T122" s="30"/>
       <c r="U122" s="30" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="V122" s="3" t="s">
-        <v>1032</v>
-      </c>
-    </row>
-    <row r="123" spans="1:22" ht="75" x14ac:dyDescent="0.25">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="123" spans="1:22" ht="90" x14ac:dyDescent="0.25">
       <c r="A123" s="17" t="s">
         <v>648</v>
       </c>
       <c r="B123" s="17" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="C123" s="19" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="D123" s="20" t="s">
         <v>405</v>
@@ -12029,7 +12050,7 @@
         <v>98</v>
       </c>
       <c r="L123" s="3" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="M123" s="15" t="s">
         <v>650</v>
@@ -12053,13 +12074,13 @@
         <v>29</v>
       </c>
       <c r="U123" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V123" s="3" t="s">
-        <v>1033</v>
-      </c>
-    </row>
-    <row r="124" spans="1:22" ht="255" x14ac:dyDescent="0.25">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="124" spans="1:22" ht="150" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>433</v>
       </c>
@@ -12067,7 +12088,7 @@
         <v>434</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D124" t="s">
         <v>38</v>
@@ -12118,13 +12139,13 @@
         <v>30</v>
       </c>
       <c r="U124" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V124" s="3" t="s">
-        <v>1034</v>
-      </c>
-    </row>
-    <row r="125" spans="1:22" s="17" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="125" spans="1:22" s="17" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>439</v>
       </c>
@@ -12178,13 +12199,13 @@
       </c>
       <c r="T125" s="30"/>
       <c r="U125" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V125" s="3" t="s">
-        <v>1019</v>
-      </c>
-    </row>
-    <row r="126" spans="1:22" ht="120" x14ac:dyDescent="0.25">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="126" spans="1:22" ht="90" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>444</v>
       </c>
@@ -12216,7 +12237,7 @@
         <v>38</v>
       </c>
       <c r="L126" s="3" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="M126" s="3" t="s">
         <v>38</v>
@@ -12240,10 +12261,10 @@
         <v>30</v>
       </c>
       <c r="U126" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V126" s="3" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="127" spans="1:22" ht="120" x14ac:dyDescent="0.25">
@@ -12302,10 +12323,10 @@
         <v>30</v>
       </c>
       <c r="U127" s="30" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="V127" s="3" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
     </row>
     <row r="128" spans="1:22" s="17" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -12343,7 +12364,7 @@
         <v>138</v>
       </c>
       <c r="L128" s="3" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="M128" s="3" t="s">
         <v>38</v>
@@ -12368,10 +12389,10 @@
       </c>
       <c r="T128" s="30"/>
       <c r="U128" s="30" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="V128" s="3" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="129" spans="1:22" s="17" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -12409,7 +12430,7 @@
         <v>38</v>
       </c>
       <c r="L129" s="3" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="M129" s="3" t="s">
         <v>457</v>
@@ -12434,13 +12455,13 @@
       </c>
       <c r="T129" s="30"/>
       <c r="U129" s="30" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="V129" s="3" t="s">
-        <v>1036</v>
-      </c>
-    </row>
-    <row r="130" spans="1:22" ht="105" x14ac:dyDescent="0.25">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="130" spans="1:22" ht="75" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>547</v>
       </c>
@@ -12475,7 +12496,7 @@
         <v>38</v>
       </c>
       <c r="L130" s="3" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="M130" s="3" t="s">
         <v>245</v>
@@ -12499,13 +12520,13 @@
         <v>29</v>
       </c>
       <c r="U130" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V130" s="3" t="s">
-        <v>979</v>
-      </c>
-    </row>
-    <row r="131" spans="1:22" ht="90" x14ac:dyDescent="0.25">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="131" spans="1:22" ht="300" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>458</v>
       </c>
@@ -12537,7 +12558,7 @@
         <v>38</v>
       </c>
       <c r="L131" s="3" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="M131" s="3" t="s">
         <v>38</v>
@@ -12561,13 +12582,13 @@
         <v>29</v>
       </c>
       <c r="U131" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V131" s="3" t="s">
-        <v>1018</v>
-      </c>
-    </row>
-    <row r="132" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="132" spans="1:22" ht="270" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>461</v>
       </c>
@@ -12623,13 +12644,13 @@
         <v>29</v>
       </c>
       <c r="U132" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V132" s="3" t="s">
-        <v>1018</v>
-      </c>
-    </row>
-    <row r="133" spans="1:22" ht="90" x14ac:dyDescent="0.25">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="133" spans="1:22" ht="120" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>466</v>
       </c>
@@ -12637,7 +12658,7 @@
         <v>467</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="D133" t="s">
         <v>38</v>
@@ -12664,7 +12685,7 @@
         <v>38</v>
       </c>
       <c r="L133" s="3" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="M133" s="3" t="s">
         <v>470</v>
@@ -12688,13 +12709,13 @@
         <v>30</v>
       </c>
       <c r="U133" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V133" s="3" t="s">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="134" spans="1:22" s="17" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="134" spans="1:22" s="17" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>219</v>
       </c>
@@ -12750,13 +12771,13 @@
       </c>
       <c r="T134" s="30"/>
       <c r="U134" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V134" s="3" t="s">
-        <v>957</v>
-      </c>
-    </row>
-    <row r="135" spans="1:22" ht="150" x14ac:dyDescent="0.25">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="135" spans="1:22" ht="90" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>471</v>
       </c>
@@ -12764,7 +12785,7 @@
         <v>472</v>
       </c>
       <c r="C135" s="19" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="D135" t="s">
         <v>38</v>
@@ -12788,7 +12809,7 @@
         <v>38</v>
       </c>
       <c r="L135" s="3" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="M135" s="3" t="s">
         <v>38</v>
@@ -12812,13 +12833,13 @@
         <v>30</v>
       </c>
       <c r="U135" s="30" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="V135" s="3" t="s">
-        <v>1042</v>
-      </c>
-    </row>
-    <row r="136" spans="1:22" ht="90" x14ac:dyDescent="0.25">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="136" spans="1:22" ht="105" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>475</v>
       </c>
@@ -12826,7 +12847,7 @@
         <v>476</v>
       </c>
       <c r="C136" s="19" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="D136" t="s">
         <v>38</v>
@@ -12850,13 +12871,13 @@
         <v>38</v>
       </c>
       <c r="L136" s="3" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="M136" s="3" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="N136" s="3" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O136" s="32" t="s">
         <v>30</v>
@@ -12874,10 +12895,10 @@
         <v>30</v>
       </c>
       <c r="U136" s="30" t="s">
+        <v>901</v>
+      </c>
+      <c r="V136" s="3" t="s">
         <v>902</v>
-      </c>
-      <c r="V136" s="3" t="s">
-        <v>903</v>
       </c>
     </row>
     <row r="137" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -12888,7 +12909,7 @@
         <v>479</v>
       </c>
       <c r="C137" s="19" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="D137" t="s">
         <v>38</v>
@@ -12912,13 +12933,13 @@
         <v>38</v>
       </c>
       <c r="L137" s="3" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="M137" s="3" t="s">
         <v>38</v>
       </c>
       <c r="N137" s="3" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="O137" s="32" t="s">
         <v>29</v>
@@ -12939,13 +12960,13 @@
         <v>15</v>
       </c>
       <c r="U137" s="30" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="V137" s="3" t="s">
-        <v>980</v>
-      </c>
-    </row>
-    <row r="138" spans="1:22" ht="165" x14ac:dyDescent="0.25">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="138" spans="1:22" ht="90" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>481</v>
       </c>
@@ -12953,7 +12974,7 @@
         <v>482</v>
       </c>
       <c r="C138" s="19" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="D138" t="s">
         <v>38</v>
@@ -12977,13 +12998,13 @@
         <v>38</v>
       </c>
       <c r="L138" s="3" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="M138" s="3" t="s">
         <v>38</v>
       </c>
       <c r="N138" s="3" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="O138" s="32" t="s">
         <v>30</v>
@@ -13001,21 +13022,21 @@
         <v>29</v>
       </c>
       <c r="U138" s="30" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="V138" s="3" t="s">
-        <v>1039</v>
-      </c>
-    </row>
-    <row r="139" spans="1:22" s="16" customFormat="1" ht="120" x14ac:dyDescent="0.25">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="139" spans="1:22" s="16" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>570</v>
       </c>
       <c r="B139" s="17" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="C139" s="19" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="D139" t="s">
         <v>38</v>
@@ -13040,7 +13061,7 @@
         <v>38</v>
       </c>
       <c r="L139" s="3" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="M139" s="3" t="s">
         <v>38</v>
@@ -13065,13 +13086,13 @@
       </c>
       <c r="T139" s="30"/>
       <c r="U139" s="30" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="V139" s="3" t="s">
-        <v>936</v>
-      </c>
-    </row>
-    <row r="140" spans="1:22" s="16" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="140" spans="1:22" s="16" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>484</v>
       </c>
@@ -13079,7 +13100,7 @@
         <v>485</v>
       </c>
       <c r="C140" s="19" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="D140" t="s">
         <v>38</v>
@@ -13104,7 +13125,7 @@
         <v>38</v>
       </c>
       <c r="L140" s="3" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="M140" s="3" t="s">
         <v>745</v>
@@ -13129,10 +13150,10 @@
       </c>
       <c r="T140" s="30"/>
       <c r="U140" s="30" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="V140" s="3" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="141" spans="1:22" ht="90" x14ac:dyDescent="0.25">
@@ -13167,7 +13188,7 @@
         <v>38</v>
       </c>
       <c r="L141" s="3" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="M141" s="3" t="s">
         <v>38</v>
@@ -13191,10 +13212,10 @@
         <v>30</v>
       </c>
       <c r="U141" s="30" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="V141" s="3" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="142" spans="1:22" ht="120" x14ac:dyDescent="0.25">
@@ -13205,7 +13226,7 @@
         <v>528</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="D142" t="s">
         <v>38</v>
@@ -13253,13 +13274,13 @@
         <v>30</v>
       </c>
       <c r="U142" s="30" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="V142" s="3" t="s">
-        <v>1038</v>
-      </c>
-    </row>
-    <row r="143" spans="1:22" ht="90" x14ac:dyDescent="0.25">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="143" spans="1:22" ht="120" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>490</v>
       </c>
@@ -13291,7 +13312,7 @@
         <v>38</v>
       </c>
       <c r="L143" s="3" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="M143" s="3" t="s">
         <v>38</v>
@@ -13313,13 +13334,13 @@
       </c>
       <c r="S143" s="33"/>
       <c r="U143" s="30" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="V143" s="3" t="s">
-        <v>1041</v>
-      </c>
-    </row>
-    <row r="144" spans="1:22" s="16" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="144" spans="1:22" s="16" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>493</v>
       </c>
@@ -13352,7 +13373,7 @@
         <v>23</v>
       </c>
       <c r="L144" s="3" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="M144" s="3" t="s">
         <v>496</v>
@@ -13377,10 +13398,10 @@
       </c>
       <c r="T144" s="30"/>
       <c r="U144" s="30" t="s">
+        <v>923</v>
+      </c>
+      <c r="V144" s="3" t="s">
         <v>924</v>
-      </c>
-      <c r="V144" s="3" t="s">
-        <v>925</v>
       </c>
     </row>
     <row r="145" spans="1:22" ht="315" x14ac:dyDescent="0.25">
@@ -13391,7 +13412,7 @@
         <v>745</v>
       </c>
       <c r="C145" s="27" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="D145" s="7" t="s">
         <v>38</v>
@@ -13413,7 +13434,7 @@
         <v>2006</v>
       </c>
       <c r="L145" s="3" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="M145" s="3" t="s">
         <v>38</v>
@@ -13433,18 +13454,73 @@
       <c r="R145" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="S145" s="33" t="s">
+      <c r="S145" s="38" t="s">
         <v>29</v>
       </c>
       <c r="T145" s="30">
         <v>30</v>
       </c>
       <c r="U145" s="32" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="V145" s="34" t="s">
-        <v>901</v>
-      </c>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="146" spans="1:22" ht="105" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B146" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>1087</v>
+      </c>
+      <c r="D146" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E146" s="1" t="s">
+        <v>1088</v>
+      </c>
+      <c r="F146" t="s">
+        <v>38</v>
+      </c>
+      <c r="H146" s="1"/>
+      <c r="I146" s="10">
+        <v>1</v>
+      </c>
+      <c r="J146">
+        <v>2025</v>
+      </c>
+      <c r="K146" t="s">
+        <v>1089</v>
+      </c>
+      <c r="L146" s="3" t="s">
+        <v>1090</v>
+      </c>
+      <c r="M146" t="s">
+        <v>1091</v>
+      </c>
+      <c r="N146" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="O146" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="P146" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q146" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="R146" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="S146" s="38"/>
+      <c r="T146" s="32"/>
+      <c r="U146" s="32"/>
+      <c r="V146" s="34"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -13693,12 +13769,13 @@
     <hyperlink ref="C140" r:id="rId242" xr:uid="{31E930C8-EAAF-4B34-8443-75427984FA75}"/>
     <hyperlink ref="C102" r:id="rId243" xr:uid="{379FD10B-9650-463A-84C0-55B4727D7D47}"/>
     <hyperlink ref="E102" r:id="rId244" xr:uid="{F803CDF1-49F8-4F15-83C4-1374EEB2B30A}"/>
+    <hyperlink ref="C146" r:id="rId245" xr:uid="{C5C87514-E810-480B-A94B-83BB9DAD7389}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId245"/>
-  <legacyDrawing r:id="rId246"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId246"/>
+  <legacyDrawing r:id="rId247"/>
   <tableParts count="1">
-    <tablePart r:id="rId247"/>
+    <tablePart r:id="rId248"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -13707,7 +13784,7 @@
           <x14:formula1>
             <xm:f>Domains!$A$2:$A$28</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:H2 G4:H53 G55:H62 G64:H69 G71:H145</xm:sqref>
+          <xm:sqref>G2:H2 G4:H53 G55:H62 G64:H69 G71:H145 G146</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -13877,15 +13954,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7e06419a-bc24-4bca-aaf1-3b90bf7d837a">
@@ -13893,6 +13961,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14100,19 +14177,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1E73802-DE0F-482B-8B75-044CD712CFB1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CBC734A-37E0-4A55-B328-89CFAE297459}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="7e06419a-bc24-4bca-aaf1-3b90bf7d837a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CBC734A-37E0-4A55-B328-89CFAE297459}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1E73802-DE0F-482B-8B75-044CD712CFB1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="7e06419a-bc24-4bca-aaf1-3b90bf7d837a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>